<commit_message>
Correção de contadores de linha e coluna. Versão final 2
</commit_message>
<xml_diff>
--- a/LL1_GrammarTable.xlsx
+++ b/LL1_GrammarTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/024519c66ae4243b/Codes/Compilers1/T1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="241" documentId="8_{936C9265-86C8-4B38-A526-30ADCF32F8C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C21AA7A2-A3FD-4CE7-8AB3-2A720B36483C}"/>
+  <xr:revisionPtr revIDLastSave="242" documentId="8_{936C9265-86C8-4B38-A526-30ADCF32F8C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C59419B5-E833-4936-875D-BFEB075D80E9}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="3" xr2:uid="{3E09A380-1B27-4448-8CF0-54497541E24D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{3E09A380-1B27-4448-8CF0-54497541E24D}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -1127,10 +1127,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1451,15 +1447,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{016D94C4-B8AC-4D3C-B46F-D5FDBE8C81C8}">
   <dimension ref="B2:F56"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.54296875" customWidth="1"/>
-    <col min="3" max="3" width="10.26953125" customWidth="1"/>
-    <col min="4" max="4" width="3.453125" customWidth="1"/>
-    <col min="5" max="5" width="31.7265625" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" customWidth="1"/>
+    <col min="4" max="4" width="3.42578125" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -1470,7 +1466,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>25</v>
       </c>
@@ -1484,7 +1480,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>26</v>
       </c>
@@ -1498,7 +1494,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>27</v>
       </c>
@@ -1512,7 +1508,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>28</v>
       </c>
@@ -1526,7 +1522,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>29</v>
       </c>
@@ -1540,7 +1536,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>30</v>
       </c>
@@ -1554,7 +1550,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>31</v>
       </c>
@@ -1568,7 +1564,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>32</v>
       </c>
@@ -1582,7 +1578,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>33</v>
       </c>
@@ -1596,7 +1592,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>34</v>
       </c>
@@ -1610,7 +1606,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>35</v>
       </c>
@@ -1624,7 +1620,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>36</v>
       </c>
@@ -1638,7 +1634,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>37</v>
       </c>
@@ -1652,7 +1648,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>38</v>
       </c>
@@ -1666,7 +1662,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>39</v>
       </c>
@@ -1680,7 +1676,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>40</v>
       </c>
@@ -1694,7 +1690,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>41</v>
       </c>
@@ -1708,7 +1704,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>42</v>
       </c>
@@ -1722,7 +1718,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>43</v>
       </c>
@@ -1736,7 +1732,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>44</v>
       </c>
@@ -1750,7 +1746,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>45</v>
       </c>
@@ -1764,7 +1760,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>46</v>
       </c>
@@ -1778,7 +1774,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>47</v>
       </c>
@@ -1792,7 +1788,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
         <v>129</v>
       </c>
@@ -1803,7 +1799,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
         <v>130</v>
       </c>
@@ -1814,7 +1810,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C28" t="s">
         <v>131</v>
       </c>
@@ -1825,7 +1821,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E29" t="b">
         <v>0</v>
       </c>
@@ -1833,7 +1829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E30" t="s">
         <v>53</v>
       </c>
@@ -1841,7 +1837,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E31" t="s">
         <v>75</v>
       </c>
@@ -1849,7 +1845,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E32" t="s">
         <v>76</v>
       </c>
@@ -1857,7 +1853,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E33" t="s">
         <v>77</v>
       </c>
@@ -1865,7 +1861,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E34" t="s">
         <v>78</v>
       </c>
@@ -1873,7 +1869,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E35" t="s">
         <v>79</v>
       </c>
@@ -1881,7 +1877,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E36" t="s">
         <v>80</v>
       </c>
@@ -1889,7 +1885,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E37" t="s">
         <v>81</v>
       </c>
@@ -1897,7 +1893,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E38" t="s">
         <v>122</v>
       </c>
@@ -1905,82 +1901,82 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E39" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="40" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E40" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="41" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E41" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="42" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E42" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="43" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E43" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="44" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E44" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="45" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E45" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="46" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E46" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="47" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E47" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="48" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E48" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="49" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="50" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E50" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="51" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E51" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="52" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="53" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E53" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="54" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E54" t="s">
         <v>123</v>
       </c>
@@ -1988,7 +1984,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="55" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E55" t="s">
         <v>124</v>
       </c>
@@ -1996,7 +1992,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="56" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
         <v>125</v>
       </c>
@@ -2012,26 +2008,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DF1DED4-D4DC-4627-8255-69DE557397B2}">
   <dimension ref="B2:BH40"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.81640625" customWidth="1"/>
-    <col min="3" max="3" width="9.1796875" customWidth="1"/>
-    <col min="4" max="4" width="30.453125" customWidth="1"/>
-    <col min="5" max="5" width="14.7265625" customWidth="1"/>
+    <col min="1" max="1" width="3.85546875" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="30.42578125" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="9" max="9" width="17.54296875" customWidth="1"/>
-    <col min="10" max="10" width="10.81640625" customWidth="1"/>
-    <col min="14" max="14" width="13.453125" customWidth="1"/>
-    <col min="22" max="22" width="21.81640625" customWidth="1"/>
+    <col min="9" max="9" width="17.5703125" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" customWidth="1"/>
+    <col min="14" max="14" width="13.42578125" customWidth="1"/>
+    <col min="22" max="22" width="21.85546875" customWidth="1"/>
     <col min="23" max="23" width="16" customWidth="1"/>
     <col min="25" max="25" width="14" customWidth="1"/>
     <col min="33" max="33" width="13" customWidth="1"/>
-    <col min="41" max="41" width="11.453125" customWidth="1"/>
-    <col min="55" max="55" width="16.54296875" customWidth="1"/>
-    <col min="56" max="56" width="18.1796875" customWidth="1"/>
+    <col min="41" max="41" width="11.42578125" customWidth="1"/>
+    <col min="55" max="55" width="16.5703125" customWidth="1"/>
+    <col min="56" max="56" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>132</v>
       </c>
@@ -2207,7 +2203,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>137</v>
       </c>
@@ -2275,7 +2271,7 @@
       <c r="BF3" s="1"/>
       <c r="BG3" s="1"/>
     </row>
-    <row r="4" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>140</v>
       </c>
@@ -2347,7 +2343,7 @@
       <c r="BF4" s="1"/>
       <c r="BG4" s="1"/>
     </row>
-    <row r="5" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>145</v>
       </c>
@@ -2415,7 +2411,7 @@
       <c r="BF5" s="1"/>
       <c r="BG5" s="1"/>
     </row>
-    <row r="6" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>148</v>
       </c>
@@ -2484,7 +2480,7 @@
       <c r="BG6" s="1"/>
       <c r="BH6" s="2"/>
     </row>
-    <row r="7" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>150</v>
       </c>
@@ -2556,7 +2552,7 @@
       <c r="BF7" s="1"/>
       <c r="BG7" s="1"/>
     </row>
-    <row r="8" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>154</v>
       </c>
@@ -2642,7 +2638,7 @@
       <c r="BF8" s="1"/>
       <c r="BG8" s="1"/>
     </row>
-    <row r="9" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>158</v>
       </c>
@@ -2718,7 +2714,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="10" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>162</v>
       </c>
@@ -2796,7 +2792,7 @@
       <c r="BF10" s="1"/>
       <c r="BG10" s="1"/>
     </row>
-    <row r="11" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>154</v>
       </c>
@@ -2884,7 +2880,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="12" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>162</v>
       </c>
@@ -2962,7 +2958,7 @@
       <c r="BF12" s="1"/>
       <c r="BG12" s="1"/>
     </row>
-    <row r="13" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>172</v>
       </c>
@@ -3030,7 +3026,7 @@
       <c r="BF13" s="1"/>
       <c r="BG13" s="1"/>
     </row>
-    <row r="14" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>174</v>
       </c>
@@ -3106,7 +3102,7 @@
       <c r="BF14" s="1"/>
       <c r="BG14" s="1"/>
     </row>
-    <row r="15" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
         <v>176</v>
       </c>
@@ -3174,7 +3170,7 @@
       <c r="BF15" s="1"/>
       <c r="BG15" s="1"/>
     </row>
-    <row r="16" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
         <v>179</v>
       </c>
@@ -3246,7 +3242,7 @@
       <c r="BF16" s="1"/>
       <c r="BG16" s="1"/>
     </row>
-    <row r="17" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>183</v>
       </c>
@@ -3316,7 +3312,7 @@
       <c r="BF17" s="1"/>
       <c r="BG17" s="1"/>
     </row>
-    <row r="18" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>187</v>
       </c>
@@ -3384,7 +3380,7 @@
       <c r="BF18" s="1"/>
       <c r="BG18" s="1"/>
     </row>
-    <row r="19" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>179</v>
       </c>
@@ -3454,7 +3450,7 @@
       <c r="BF19" s="1"/>
       <c r="BG19" s="1"/>
     </row>
-    <row r="20" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>174</v>
       </c>
@@ -3530,7 +3526,7 @@
       <c r="BF20" s="1"/>
       <c r="BG20" s="1"/>
     </row>
-    <row r="21" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
         <v>141</v>
       </c>
@@ -3598,7 +3594,7 @@
       <c r="BF21" s="1"/>
       <c r="BG21" s="1"/>
     </row>
-    <row r="22" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>200</v>
       </c>
@@ -3678,7 +3674,7 @@
       <c r="BF22" s="1"/>
       <c r="BG22" s="1"/>
     </row>
-    <row r="23" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>203</v>
       </c>
@@ -3766,7 +3762,7 @@
       <c r="BF23" s="1"/>
       <c r="BG23" s="1"/>
     </row>
-    <row r="24" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
         <v>200</v>
       </c>
@@ -3846,7 +3842,7 @@
       <c r="BF24" s="1"/>
       <c r="BG24" s="1"/>
     </row>
-    <row r="25" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
         <v>215</v>
       </c>
@@ -3920,7 +3916,7 @@
       <c r="BF25" s="1"/>
       <c r="BG25" s="1"/>
     </row>
-    <row r="26" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
         <v>221</v>
       </c>
@@ -3990,7 +3986,7 @@
       <c r="BF26" s="1"/>
       <c r="BG26" s="1"/>
     </row>
-    <row r="27" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
         <v>226</v>
       </c>
@@ -4060,7 +4056,7 @@
       <c r="BF27" s="1"/>
       <c r="BG27" s="1"/>
     </row>
-    <row r="28" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>231</v>
       </c>
@@ -4174,7 +4170,7 @@
       </c>
       <c r="BG28" s="1"/>
     </row>
-    <row r="29" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
         <v>234</v>
       </c>
@@ -4268,7 +4264,7 @@
       <c r="BF29" s="1"/>
       <c r="BG29" s="1"/>
     </row>
-    <row r="30" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
         <v>243</v>
       </c>
@@ -4382,7 +4378,7 @@
       </c>
       <c r="BG30" s="1"/>
     </row>
-    <row r="31" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>246</v>
       </c>
@@ -4468,7 +4464,7 @@
       </c>
       <c r="BG31" s="1"/>
     </row>
-    <row r="32" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
         <v>252</v>
       </c>
@@ -4568,7 +4564,7 @@
       <c r="BF32" s="1"/>
       <c r="BG32" s="1"/>
     </row>
-    <row r="33" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
         <v>247</v>
       </c>
@@ -4650,7 +4646,7 @@
       </c>
       <c r="BG33" s="1"/>
     </row>
-    <row r="34" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
         <v>260</v>
       </c>
@@ -4758,7 +4754,7 @@
       <c r="BF34" s="1"/>
       <c r="BG34" s="1"/>
     </row>
-    <row r="35" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
         <v>247</v>
       </c>
@@ -4840,7 +4836,7 @@
       </c>
       <c r="BG35" s="1"/>
     </row>
-    <row r="36" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
         <v>276</v>
       </c>
@@ -4952,7 +4948,7 @@
       <c r="BF36" s="1"/>
       <c r="BG36" s="1"/>
     </row>
-    <row r="37" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
         <v>176</v>
       </c>
@@ -5020,7 +5016,7 @@
       <c r="BF37" s="1"/>
       <c r="BG37" s="1"/>
     </row>
-    <row r="38" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
         <v>282</v>
       </c>
@@ -5130,7 +5126,7 @@
       <c r="BF38" s="1"/>
       <c r="BG38" s="1"/>
     </row>
-    <row r="39" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
         <v>286</v>
       </c>
@@ -5234,7 +5230,7 @@
       </c>
       <c r="BG39" s="1"/>
     </row>
-    <row r="40" spans="2:59" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B40" s="1" t="s">
         <v>179</v>
       </c>
@@ -5314,16 +5310,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB16E5C9-8C5D-43AE-B1A8-08D490655B6A}">
   <dimension ref="A1:BE39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="27.7265625" customWidth="1"/>
-    <col min="3" max="3" width="11.7265625" customWidth="1"/>
-    <col min="4" max="4" width="12.81640625" customWidth="1"/>
-    <col min="7" max="7" width="15.1796875" customWidth="1"/>
-    <col min="54" max="54" width="17.81640625" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" customWidth="1"/>
+    <col min="54" max="54" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:57" x14ac:dyDescent="0.25">
       <c r="B1" s="7" t="str">
         <f>'LL1 Parser Table'!D2</f>
         <v>Nonterminal</v>
@@ -5549,7 +5545,7 @@
         <v>$</v>
       </c>
     </row>
-    <row r="2" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5778,7 +5774,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="3" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -6007,7 +6003,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="4" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -6236,7 +6232,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="5" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -6465,7 +6461,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="6" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -6694,7 +6690,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="7" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -6923,7 +6919,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="8" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -7152,7 +7148,7 @@
         <v>BlocoVariaveis -&gt; ''</v>
       </c>
     </row>
-    <row r="9" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -7381,7 +7377,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="10" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -7610,7 +7606,7 @@
         <v>DeclaracoesBonus -&gt; ''</v>
       </c>
     </row>
-    <row r="11" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -7839,7 +7835,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="12" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -8068,7 +8064,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="13" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -8297,7 +8293,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="14" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -8526,7 +8522,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="15" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -8755,7 +8751,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="16" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -8984,7 +8980,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="17" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -9213,7 +9209,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="18" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -9442,7 +9438,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="19" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -9671,7 +9667,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="20" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -9900,7 +9896,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="21" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -10129,7 +10125,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="22" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -10358,7 +10354,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="23" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -10587,7 +10583,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="24" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -10816,7 +10812,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="25" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -11045,7 +11041,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="26" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -11274,7 +11270,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="27" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -11503,7 +11499,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="28" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -11732,7 +11728,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="29" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -11961,7 +11957,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="30" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -12190,7 +12186,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="31" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -12419,7 +12415,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="32" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -12648,7 +12644,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="33" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -12877,7 +12873,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="34" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -13106,7 +13102,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="35" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -13335,7 +13331,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="36" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -13564,7 +13560,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="37" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -13793,7 +13789,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="38" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -14022,7 +14018,7 @@
         <v>ERRO</v>
       </c>
     </row>
-    <row r="39" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -14259,14 +14255,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EBCDFE9-93B7-427D-AA82-3D202CB3F68F}">
   <dimension ref="B2:BP92"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.26953125" customWidth="1"/>
-    <col min="5" max="5" width="19.54296875" customWidth="1"/>
-    <col min="8" max="8" width="97.453125" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
+    <col min="8" max="8" width="104.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>134</v>
       </c>
@@ -14451,7 +14447,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>25</v>
       </c>
@@ -14471,7 +14467,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>28</v>
       </c>
@@ -14491,7 +14487,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>29</v>
       </c>
@@ -14511,7 +14507,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>30</v>
       </c>
@@ -14531,7 +14527,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>31</v>
       </c>
@@ -14551,7 +14547,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>32</v>
       </c>
@@ -14571,7 +14567,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>26</v>
       </c>
@@ -14591,7 +14587,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>34</v>
       </c>
@@ -14611,7 +14607,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>165</v>
       </c>
@@ -14631,7 +14627,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>169</v>
       </c>
@@ -14651,7 +14647,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>36</v>
       </c>
@@ -14671,7 +14667,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>35</v>
       </c>
@@ -14691,7 +14687,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>33</v>
       </c>
@@ -14711,7 +14707,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="2:68" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:68" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>180</v>
       </c>
@@ -14731,7 +14727,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>37</v>
       </c>
@@ -14751,7 +14747,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>38</v>
       </c>
@@ -14771,7 +14767,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>190</v>
       </c>
@@ -14791,7 +14787,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>39</v>
       </c>
@@ -14811,7 +14807,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>27</v>
       </c>
@@ -14831,7 +14827,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>40</v>
       </c>
@@ -14851,7 +14847,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>204</v>
       </c>
@@ -14871,7 +14867,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>41</v>
       </c>
@@ -14891,7 +14887,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>216</v>
       </c>
@@ -14911,7 +14907,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>223</v>
       </c>
@@ -14931,7 +14927,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>228</v>
       </c>
@@ -14951,7 +14947,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>44</v>
       </c>
@@ -14971,7 +14967,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>235</v>
       </c>
@@ -14991,7 +14987,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>45</v>
       </c>
@@ -15011,7 +15007,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>248</v>
       </c>
@@ -15031,7 +15027,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>253</v>
       </c>
@@ -15051,7 +15047,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>46</v>
       </c>
@@ -15071,7 +15067,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>261</v>
       </c>
@@ -15091,7 +15087,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>47</v>
       </c>
@@ -15111,7 +15107,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>277</v>
       </c>
@@ -15131,7 +15127,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>43</v>
       </c>
@@ -15151,7 +15147,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>283</v>
       </c>
@@ -15171,7 +15167,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>42</v>
       </c>
@@ -15191,7 +15187,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>289</v>
       </c>
@@ -15211,7 +15207,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E41" t="s">
         <v>96</v>
       </c>
@@ -15225,7 +15221,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E42" t="s">
         <v>80</v>
       </c>
@@ -15239,7 +15235,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E43" t="s">
         <v>79</v>
       </c>
@@ -15253,7 +15249,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E44" t="s">
         <v>97</v>
       </c>
@@ -15267,7 +15263,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B45" t="str">
         <f>UPPER(B3)</f>
         <v>PROGRAMA</v>
@@ -15289,7 +15285,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B46" t="str">
         <f t="shared" ref="B46:B82" si="0">UPPER(B4)</f>
         <v>PROCEDIMENTOFUNCAO</v>
@@ -15311,7 +15307,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B47" t="str">
         <f t="shared" si="0"/>
         <v>DECLARAPROCEDIMENTO</v>
@@ -15333,7 +15329,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B48" t="str">
         <f t="shared" si="0"/>
         <v>DECLARAFUNCAO</v>
@@ -15355,7 +15351,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B49" t="str">
         <f t="shared" si="0"/>
         <v>PARAMETROS</v>
@@ -15377,7 +15373,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B50" t="str">
         <f t="shared" si="0"/>
         <v>DECLARAPARAMETROS</v>
@@ -15399,7 +15395,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B51" t="str">
         <f t="shared" si="0"/>
         <v>BLOCOVARIAVEIS</v>
@@ -15421,7 +15417,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B52" t="str">
         <f t="shared" si="0"/>
         <v>DECLARACOES</v>
@@ -15443,7 +15439,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B53" t="str">
         <f t="shared" si="0"/>
         <v>DECLARACOESBONUS</v>
@@ -15465,7 +15461,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B54" t="str">
         <f t="shared" si="0"/>
         <v>DECLARATIONS</v>
@@ -15487,7 +15483,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" t="str">
         <f t="shared" si="0"/>
         <v>DECLARATIPO</v>
@@ -15509,7 +15505,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" t="str">
         <f t="shared" si="0"/>
         <v>DECLARAVARIAVEIS</v>
@@ -15531,7 +15527,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" t="str">
         <f t="shared" si="0"/>
         <v>DECLARAIDENTIFICADOR</v>
@@ -15553,7 +15549,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" t="str">
         <f>UPPER(B16)</f>
         <v>DECLARAIDENTIFICADORBONUS</v>
@@ -15569,7 +15565,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="59" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B59" t="str">
         <f t="shared" si="0"/>
         <v>VETORMATRIZ</v>
@@ -15585,7 +15581,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="60" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B60" t="str">
         <f t="shared" si="0"/>
         <v>DIMENSAO</v>
@@ -15601,7 +15597,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B61" t="str">
         <f t="shared" si="0"/>
         <v>DIMENSAOBONUS</v>
@@ -15617,7 +15613,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" t="str">
         <f t="shared" si="0"/>
         <v>TIPOBASICO</v>
@@ -15633,7 +15629,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="63" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" t="str">
         <f t="shared" si="0"/>
         <v>BLOCOCOMANDOS</v>
@@ -15649,7 +15645,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="64" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" t="str">
         <f t="shared" si="0"/>
         <v>LISTACOMANDOS</v>
@@ -15665,7 +15661,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" t="str">
         <f t="shared" si="0"/>
         <v>LISTACOMANDOSBONUS</v>
@@ -15681,7 +15677,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="66" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B66" t="str">
         <f t="shared" si="0"/>
         <v>COMANDOS</v>
@@ -15697,7 +15693,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B67" t="str">
         <f t="shared" si="0"/>
         <v>COMMANDSIDENTIFIER</v>
@@ -15713,7 +15709,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="68" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B68" t="str">
         <f t="shared" si="0"/>
         <v>ELSEIF</v>
@@ -15729,7 +15725,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="69" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B69" t="str">
         <f t="shared" si="0"/>
         <v>STEPFOR</v>
@@ -15745,7 +15741,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="70" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" t="str">
         <f>UPPER(B28)</f>
         <v>EXPRESSAO</v>
@@ -15761,7 +15757,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B71" t="str">
         <f t="shared" si="0"/>
         <v>EXPRESSAONEW</v>
@@ -15777,7 +15773,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="72" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B72" t="str">
         <f t="shared" si="0"/>
         <v>EXPRESSAOSIMPLES</v>
@@ -15793,7 +15789,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="73" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B73" t="str">
         <f t="shared" si="0"/>
         <v>SIGNAL</v>
@@ -15809,7 +15805,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="74" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B74" t="str">
         <f t="shared" si="0"/>
         <v>EXPRESSAOSIMPLESNEW</v>
@@ -15825,7 +15821,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="75" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B75" t="str">
         <f t="shared" si="0"/>
         <v>TERMO</v>
@@ -15841,7 +15837,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="76" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B76" t="str">
         <f t="shared" si="0"/>
         <v>TERMONEW</v>
@@ -15857,7 +15853,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="77" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B77" t="str">
         <f t="shared" si="0"/>
         <v>FATOR</v>
@@ -15873,7 +15869,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="78" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B78" t="str">
         <f t="shared" si="0"/>
         <v>IDENTIFIERVARIABLE</v>
@@ -15889,7 +15885,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="79" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B79" t="str">
         <f>UPPER(B37)</f>
         <v>VARIAVEL</v>
@@ -15905,7 +15901,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="80" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B80" t="str">
         <f t="shared" si="0"/>
         <v>VARIABLEEXP</v>
@@ -15921,7 +15917,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="81" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B81" t="str">
         <f>UPPER(B39)</f>
         <v>EXPRITER</v>
@@ -15937,7 +15933,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="82" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" t="str">
         <f t="shared" si="0"/>
         <v>EXPRITERBONUS</v>
@@ -15953,7 +15949,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="83" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H83" t="s">
         <v>268</v>
       </c>
@@ -15961,7 +15957,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="84" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H84" t="s">
         <v>279</v>
       </c>
@@ -15969,7 +15965,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="85" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H85" t="s">
         <v>278</v>
       </c>
@@ -15977,7 +15973,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="86" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H86" t="s">
         <v>281</v>
       </c>
@@ -15985,7 +15981,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="87" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H87" t="s">
         <v>285</v>
       </c>
@@ -15993,7 +15989,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="88" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H88" t="s">
         <v>284</v>
       </c>
@@ -16001,7 +15997,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="89" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H89" t="s">
         <v>288</v>
       </c>
@@ -16009,7 +16005,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="90" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H90" t="s">
         <v>291</v>
       </c>
@@ -16017,7 +16013,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="91" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H91" t="s">
         <v>290</v>
       </c>
@@ -16025,7 +16021,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="92" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H92" t="s">
         <v>295</v>
       </c>
@@ -16042,13 +16038,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2ECEC07-E9AF-435A-9FFF-A768E1DB8FB5}">
   <dimension ref="A1:BE40"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.6328125" customWidth="1"/>
-    <col min="54" max="54" width="12.453125" customWidth="1"/>
+    <col min="1" max="1" width="27.5703125" customWidth="1"/>
+    <col min="54" max="54" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:57" x14ac:dyDescent="0.25">
       <c r="C1" t="str" cm="1">
         <f t="array" ref="C1:BE1">TRANSPOSE(Labels!E3:E57)</f>
         <v>algoritmo</v>
@@ -16216,7 +16212,7 @@
         <v>$</v>
       </c>
     </row>
-    <row r="2" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:57" x14ac:dyDescent="0.25">
       <c r="C2">
         <f>VLOOKUP(Format1!C1,Labels!$E$3:$F$57,2,FALSE)</f>
         <v>1</v>
@@ -16437,7 +16433,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A3" t="str" cm="1">
         <f t="array" ref="A3:B40">Labels!B3:C40</f>
         <v>Programa</v>
@@ -16666,7 +16662,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <v>ProcedimentoFuncao</v>
       </c>
@@ -16894,7 +16890,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <v>DeclaraProcedimento</v>
       </c>
@@ -17122,7 +17118,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <v>DeclaraFuncao</v>
       </c>
@@ -17350,7 +17346,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <v>Parametros</v>
       </c>
@@ -17578,7 +17574,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <v>DeclaraParametros</v>
       </c>
@@ -17806,7 +17802,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <v>BlocoVariaveis</v>
       </c>
@@ -18034,7 +18030,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="10" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <v>Declaracoes</v>
       </c>
@@ -18262,7 +18258,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <v>DeclaracoesBonus</v>
       </c>
@@ -18490,7 +18486,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="12" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <v>Declarations</v>
       </c>
@@ -18718,7 +18714,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <v>DeclaraTipo</v>
       </c>
@@ -18946,7 +18942,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <v>DeclaraVariaveis</v>
       </c>
@@ -19174,7 +19170,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <v>DeclaraIdentificador</v>
       </c>
@@ -19402,7 +19398,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <v>DeclaraIdentificadorBonus</v>
       </c>
@@ -19630,7 +19626,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <v>VetorMatriz</v>
       </c>
@@ -19858,7 +19854,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <v>Dimensao</v>
       </c>
@@ -20086,7 +20082,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <v>DimensaoBonus</v>
       </c>
@@ -20314,7 +20310,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <v>TipoBasico</v>
       </c>
@@ -20542,7 +20538,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <v>BlocoComandos</v>
       </c>
@@ -20770,7 +20766,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <v>ListaComandos</v>
       </c>
@@ -20998,7 +20994,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <v>ListaComandosBonus</v>
       </c>
@@ -21226,7 +21222,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <v>Comandos</v>
       </c>
@@ -21454,7 +21450,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <v>CommandsIdentifier</v>
       </c>
@@ -21682,7 +21678,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <v>ElseIf</v>
       </c>
@@ -21910,7 +21906,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <v>StepFor</v>
       </c>
@@ -22138,7 +22134,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <v>Expressao</v>
       </c>
@@ -22366,7 +22362,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="29" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <v>ExpressaoNew</v>
       </c>
@@ -22594,7 +22590,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="30" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <v>ExpressaoSimples</v>
       </c>
@@ -22822,7 +22818,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <v>Signal</v>
       </c>
@@ -23050,7 +23046,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <v>ExpressaoSimplesNew</v>
       </c>
@@ -23278,7 +23274,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="33" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <v>Termo</v>
       </c>
@@ -23506,7 +23502,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <v>TermoNew</v>
       </c>
@@ -23734,7 +23730,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <v>Fator</v>
       </c>
@@ -23962,7 +23958,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <v>IdentifierVariable</v>
       </c>
@@ -24190,7 +24186,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <v>Variavel</v>
       </c>
@@ -24418,7 +24414,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <v>VariableExp</v>
       </c>
@@ -24646,7 +24642,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="39" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <v>ExprIter</v>
       </c>
@@ -24874,7 +24870,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:57" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <v>ExprIterBonus</v>
       </c>

</xml_diff>